<commit_message>
change schema on renaksi output
</commit_message>
<xml_diff>
--- a/public/template_import/template_import_tematik.xlsx
+++ b/public/template_import/template_import_tematik.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="70">
   <si>
     <t>Tema</t>
   </si>
@@ -174,24 +174,6 @@
     <t>contoh satuan output1</t>
   </si>
   <si>
-    <t>contoh_target1_tw1</t>
-  </si>
-  <si>
-    <t>contoh_target1_tw2</t>
-  </si>
-  <si>
-    <t>contoh_target1_tw3</t>
-  </si>
-  <si>
-    <t>contoh_target1_tw4</t>
-  </si>
-  <si>
-    <t>contoh_target1_total</t>
-  </si>
-  <si>
-    <t>contoh anggaran1</t>
-  </si>
-  <si>
     <t>Perencanaan dan Penganggaran</t>
   </si>
   <si>
@@ -201,24 +183,6 @@
     <t>pelaksana</t>
   </si>
   <si>
-    <t>contoh_realisasi_target1_tw1</t>
-  </si>
-  <si>
-    <t>contoh_realisasi_target1_tw2</t>
-  </si>
-  <si>
-    <t>contoh_realisasi_target1_tw3</t>
-  </si>
-  <si>
-    <t>contoh_realisasi_target1_tw4</t>
-  </si>
-  <si>
-    <t>contoh_realisasi_target1_total</t>
-  </si>
-  <si>
-    <t>contoh_realisasi_anggaran1_total</t>
-  </si>
-  <si>
     <t>Realisasi Investasi</t>
   </si>
   <si>
@@ -231,24 +195,6 @@
     <t>contoh satuan output2</t>
   </si>
   <si>
-    <t>contoh_target2_tw1</t>
-  </si>
-  <si>
-    <t>contoh_target2_tw2</t>
-  </si>
-  <si>
-    <t>contoh_target2_tw3</t>
-  </si>
-  <si>
-    <t>contoh_target2_tw4</t>
-  </si>
-  <si>
-    <t>contoh_target2_total</t>
-  </si>
-  <si>
-    <t>contoh anggaran2</t>
-  </si>
-  <si>
     <t>Proses Bisnis dan SOP</t>
   </si>
   <si>
@@ -256,24 +202,6 @@
   </si>
   <si>
     <t>pelaksana2</t>
-  </si>
-  <si>
-    <t>contoh_realisasi_target2_tw1</t>
-  </si>
-  <si>
-    <t>contoh_realisasi_target2_tw2</t>
-  </si>
-  <si>
-    <t>contoh_realisasi_target2_tw3</t>
-  </si>
-  <si>
-    <t>contoh_realisasi_target2_tw4</t>
-  </si>
-  <si>
-    <t>contoh_realisasi_target2_total</t>
-  </si>
-  <si>
-    <t>contoh_realisasi_anggaran2_total</t>
   </si>
   <si>
     <t>Digitalisasi Pemerintahan</t>
@@ -305,10 +233,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="4">
+    <numFmt numFmtId="41" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;_-;_-@_-"/>
+    <numFmt numFmtId="44" formatCode="_-&quot;£&quot;* #,##0.00_-;\-&quot;£&quot;* #,##0.00_-;_-&quot;£&quot;* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="42" formatCode="_-&quot;£&quot;* #,##0_-;\-&quot;£&quot;* #,##0_-;_-&quot;£&quot;* &quot;-&quot;_-;_-@_-"/>
-    <numFmt numFmtId="41" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;_-;_-@_-"/>
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="44" formatCode="_-&quot;£&quot;* #,##0.00_-;\-&quot;£&quot;* #,##0.00_-;_-&quot;£&quot;* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
   <fonts count="22">
     <font>
@@ -323,18 +251,40 @@
       <charset val="134"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <u/>
       <sz val="11"/>
-      <color rgb="FF0000FF"/>
+      <color rgb="FF800080"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -355,19 +305,27 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF9C6500"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="11"/>
       <color rgb="FF9C0006"/>
       <name val="Calibri"/>
@@ -375,33 +333,11 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <b/>
       <sz val="11"/>
       <color theme="3"/>
       <name val="Calibri"/>
       <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -413,62 +349,54 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <b/>
       <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
       <color rgb="FF3F3F3F"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -483,187 +411,187 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="6" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFA5A5A5"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="9" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -686,41 +614,13 @@
       <diagonal/>
     </border>
     <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
       </top>
       <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
+        <color theme="4"/>
       </bottom>
       <diagonal/>
     </border>
@@ -736,6 +636,30 @@
       </top>
       <bottom style="thin">
         <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
       </bottom>
       <diagonal/>
     </border>
@@ -757,168 +681,172 @@
     <border>
       <left/>
       <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
       </bottom>
       <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="7" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="24" borderId="8" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="17" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="15" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="10" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="28" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="10" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="2" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -1437,55 +1365,55 @@
       <c r="S2" t="s">
         <v>51</v>
       </c>
-      <c r="T2" t="s">
+      <c r="T2">
+        <v>1</v>
+      </c>
+      <c r="U2">
+        <v>1</v>
+      </c>
+      <c r="V2">
+        <v>1</v>
+      </c>
+      <c r="W2">
+        <v>1</v>
+      </c>
+      <c r="X2">
+        <v>4</v>
+      </c>
+      <c r="Y2">
+        <v>100</v>
+      </c>
+      <c r="Z2" t="s">
         <v>52</v>
       </c>
-      <c r="U2" t="s">
+      <c r="AA2" t="s">
         <v>53</v>
       </c>
-      <c r="V2" t="s">
+      <c r="AB2" t="s">
         <v>54</v>
       </c>
-      <c r="W2" t="s">
-        <v>55</v>
-      </c>
-      <c r="X2" t="s">
-        <v>56</v>
-      </c>
-      <c r="Y2" t="s">
-        <v>57</v>
-      </c>
-      <c r="Z2" t="s">
-        <v>58</v>
-      </c>
-      <c r="AA2" t="s">
-        <v>59</v>
-      </c>
-      <c r="AB2" t="s">
-        <v>60</v>
-      </c>
-      <c r="AC2" t="s">
-        <v>61</v>
-      </c>
-      <c r="AD2" t="s">
-        <v>62</v>
-      </c>
-      <c r="AE2" t="s">
-        <v>63</v>
-      </c>
-      <c r="AF2" t="s">
-        <v>64</v>
-      </c>
-      <c r="AG2" t="s">
-        <v>65</v>
-      </c>
-      <c r="AH2" t="s">
-        <v>66</v>
+      <c r="AC2">
+        <v>1</v>
+      </c>
+      <c r="AD2">
+        <v>1</v>
+      </c>
+      <c r="AE2">
+        <v>1</v>
+      </c>
+      <c r="AF2">
+        <v>1</v>
+      </c>
+      <c r="AG2">
+        <v>4</v>
+      </c>
+      <c r="AH2">
+        <v>100</v>
       </c>
     </row>
     <row r="3" spans="1:34">
       <c r="A3" t="s">
-        <v>67</v>
+        <v>55</v>
       </c>
       <c r="B3" t="s">
         <v>35</v>
@@ -1533,58 +1461,58 @@
         <v>41</v>
       </c>
       <c r="Q3" t="s">
-        <v>68</v>
+        <v>56</v>
       </c>
       <c r="R3" t="s">
-        <v>69</v>
+        <v>57</v>
       </c>
       <c r="S3" t="s">
-        <v>70</v>
-      </c>
-      <c r="T3" t="s">
-        <v>71</v>
-      </c>
-      <c r="U3" t="s">
-        <v>72</v>
-      </c>
-      <c r="V3" t="s">
-        <v>73</v>
-      </c>
-      <c r="W3" t="s">
-        <v>74</v>
-      </c>
-      <c r="X3" t="s">
-        <v>75</v>
-      </c>
-      <c r="Y3" t="s">
-        <v>76</v>
+        <v>58</v>
+      </c>
+      <c r="T3">
+        <v>2</v>
+      </c>
+      <c r="U3">
+        <v>2</v>
+      </c>
+      <c r="V3">
+        <v>2</v>
+      </c>
+      <c r="W3">
+        <v>2</v>
+      </c>
+      <c r="X3">
+        <v>8</v>
+      </c>
+      <c r="Y3">
+        <v>100</v>
       </c>
       <c r="Z3" t="s">
-        <v>77</v>
+        <v>59</v>
       </c>
       <c r="AA3" t="s">
-        <v>78</v>
+        <v>60</v>
       </c>
       <c r="AB3" t="s">
-        <v>79</v>
-      </c>
-      <c r="AC3" t="s">
-        <v>80</v>
-      </c>
-      <c r="AD3" t="s">
-        <v>81</v>
-      </c>
-      <c r="AE3" t="s">
-        <v>82</v>
-      </c>
-      <c r="AF3" t="s">
-        <v>83</v>
-      </c>
-      <c r="AG3" t="s">
-        <v>84</v>
-      </c>
-      <c r="AH3" t="s">
-        <v>85</v>
+        <v>61</v>
+      </c>
+      <c r="AC3">
+        <v>1</v>
+      </c>
+      <c r="AD3">
+        <v>1</v>
+      </c>
+      <c r="AE3">
+        <v>1</v>
+      </c>
+      <c r="AF3">
+        <v>1</v>
+      </c>
+      <c r="AG3">
+        <v>4</v>
+      </c>
+      <c r="AH3">
+        <v>100</v>
       </c>
     </row>
   </sheetData>
@@ -1622,22 +1550,22 @@
     </row>
     <row r="3" spans="1:1">
       <c r="A3" s="2" t="s">
-        <v>67</v>
+        <v>55</v>
       </c>
     </row>
     <row r="4" spans="1:1">
       <c r="A4" s="2" t="s">
-        <v>86</v>
+        <v>62</v>
       </c>
     </row>
     <row r="5" spans="1:1">
       <c r="A5" s="2" t="s">
-        <v>87</v>
+        <v>63</v>
       </c>
     </row>
     <row r="6" spans="1:1">
       <c r="A6" s="2" t="s">
-        <v>88</v>
+        <v>64</v>
       </c>
     </row>
   </sheetData>
@@ -1662,37 +1590,37 @@
     </row>
     <row r="2" spans="1:1">
       <c r="A2" s="2" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
     </row>
     <row r="3" spans="1:1">
       <c r="A3" s="2" t="s">
-        <v>77</v>
+        <v>59</v>
       </c>
     </row>
     <row r="4" spans="1:1">
       <c r="A4" s="2" t="s">
-        <v>89</v>
+        <v>65</v>
       </c>
     </row>
     <row r="5" spans="1:1">
       <c r="A5" s="2" t="s">
-        <v>90</v>
+        <v>66</v>
       </c>
     </row>
     <row r="6" spans="1:1">
       <c r="A6" s="2" t="s">
-        <v>91</v>
+        <v>67</v>
       </c>
     </row>
     <row r="7" spans="1:1">
       <c r="A7" s="2" t="s">
-        <v>92</v>
+        <v>68</v>
       </c>
     </row>
     <row r="8" spans="1:1">
       <c r="A8" s="2" t="s">
-        <v>93</v>
+        <v>69</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add column keterangan on output renaksi
</commit_message>
<xml_diff>
--- a/public/template_import/template_import_tematik.xlsx
+++ b/public/template_import/template_import_tematik.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="30240" windowHeight="14640" tabRatio="500"/>
+    <workbookView windowWidth="30240" windowHeight="13960" tabRatio="500"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="73">
   <si>
     <t>Tema</t>
   </si>
@@ -120,6 +120,9 @@
     <t>Realisasi Anggaran</t>
   </si>
   <si>
+    <t>Catatan Monev</t>
+  </si>
+  <si>
     <t>Pengentasan Kemiskinan</t>
   </si>
   <si>
@@ -183,6 +186,9 @@
     <t>pelaksana</t>
   </si>
   <si>
+    <t>catatan1</t>
+  </si>
+  <si>
     <t>Realisasi Investasi</t>
   </si>
   <si>
@@ -202,6 +208,9 @@
   </si>
   <si>
     <t>pelaksana2</t>
+  </si>
+  <si>
+    <t>catatan 2</t>
   </si>
   <si>
     <t>Digitalisasi Pemerintahan</t>
@@ -233,10 +242,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="4">
+    <numFmt numFmtId="44" formatCode="_-&quot;£&quot;* #,##0.00_-;\-&quot;£&quot;* #,##0.00_-;_-&quot;£&quot;* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="41" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;_-;_-@_-"/>
-    <numFmt numFmtId="44" formatCode="_-&quot;£&quot;* #,##0.00_-;\-&quot;£&quot;* #,##0.00_-;_-&quot;£&quot;* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="42" formatCode="_-&quot;£&quot;* #,##0_-;\-&quot;£&quot;* #,##0_-;_-&quot;£&quot;* &quot;-&quot;_-;_-@_-"/>
-    <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
   <fonts count="22">
     <font>
@@ -251,6 +260,14 @@
       <charset val="134"/>
     </font>
     <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -258,8 +275,113 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -273,28 +395,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <b/>
       <sz val="15"/>
       <color theme="3"/>
@@ -304,103 +404,12 @@
     </font>
     <font>
       <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="18"/>
       <color theme="3"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
   <fills count="33">
     <fill>
@@ -411,37 +420,163 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="8" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -453,145 +588,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="8"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="8" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -602,26 +611,6 @@
       <right/>
       <top/>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -642,9 +631,41 @@
     <border>
       <left/>
       <right/>
-      <top/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
       <bottom style="double">
-        <color rgb="FFFF8001"/>
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
       </bottom>
       <diagonal/>
     </border>
@@ -664,21 +685,6 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left/>
       <right/>
       <top/>
@@ -688,165 +694,168 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
       </bottom>
       <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="7" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="24" borderId="8" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="17" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="4" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="15" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="13" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -1174,7 +1183,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:AH3"/>
+  <dimension ref="A1:AI3"/>
   <sheetFormatPr defaultColWidth="8.4453125" defaultRowHeight="14" outlineLevelRow="2"/>
   <cols>
     <col min="1" max="1" width="29.6640625" customWidth="1"/>
@@ -1203,7 +1212,7 @@
     <col min="34" max="34" width="20.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:34">
+    <row r="1" spans="1:35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1306,64 +1315,67 @@
       <c r="AH1" s="1" t="s">
         <v>33</v>
       </c>
+      <c r="AI1" s="1" t="s">
+        <v>34</v>
+      </c>
     </row>
-    <row r="2" spans="1:34">
+    <row r="2" spans="1:35">
       <c r="A2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="E2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="F2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="G2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="H2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="I2" t="s">
+        <v>43</v>
+      </c>
+      <c r="J2" t="s">
+        <v>44</v>
+      </c>
+      <c r="K2" t="s">
+        <v>45</v>
+      </c>
+      <c r="L2" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="M2" t="s">
+        <v>47</v>
+      </c>
+      <c r="N2" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="O2" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="P2" t="s">
         <v>42</v>
       </c>
-      <c r="J2" t="s">
-        <v>43</v>
-      </c>
-      <c r="K2" t="s">
-        <v>44</v>
-      </c>
-      <c r="L2" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="M2" t="s">
-        <v>46</v>
-      </c>
-      <c r="N2" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="O2" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="P2" t="s">
-        <v>41</v>
-      </c>
       <c r="Q2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="R2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="S2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="T2">
         <v>1</v>
@@ -1384,13 +1396,13 @@
         <v>100</v>
       </c>
       <c r="Z2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="AA2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="AB2" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="AC2">
         <v>1</v>
@@ -1410,64 +1422,67 @@
       <c r="AH2">
         <v>100</v>
       </c>
+      <c r="AI2" t="s">
+        <v>56</v>
+      </c>
     </row>
-    <row r="3" spans="1:34">
+    <row r="3" spans="1:35">
       <c r="A3" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B3" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C3" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="E3" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="F3" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="G3" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="H3" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="I3" t="s">
+        <v>43</v>
+      </c>
+      <c r="J3" t="s">
+        <v>44</v>
+      </c>
+      <c r="K3" t="s">
+        <v>45</v>
+      </c>
+      <c r="L3" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="M3" t="s">
+        <v>47</v>
+      </c>
+      <c r="N3" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="O3" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="P3" t="s">
         <v>42</v>
       </c>
-      <c r="J3" t="s">
-        <v>43</v>
-      </c>
-      <c r="K3" t="s">
-        <v>44</v>
-      </c>
-      <c r="L3" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="M3" t="s">
-        <v>46</v>
-      </c>
-      <c r="N3" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="O3" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="P3" t="s">
-        <v>41</v>
-      </c>
       <c r="Q3" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="R3" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="S3" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="T3">
         <v>2</v>
@@ -1488,13 +1503,13 @@
         <v>100</v>
       </c>
       <c r="Z3" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="AA3" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="AB3" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="AC3">
         <v>1</v>
@@ -1513,6 +1528,9 @@
       </c>
       <c r="AH3">
         <v>100</v>
+      </c>
+      <c r="AI3" t="s">
+        <v>64</v>
       </c>
     </row>
   </sheetData>
@@ -1545,27 +1563,27 @@
     </row>
     <row r="2" spans="1:1">
       <c r="A2" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="3" spans="1:1">
       <c r="A3" s="2" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
     </row>
     <row r="4" spans="1:1">
       <c r="A4" s="2" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
     </row>
     <row r="5" spans="1:1">
       <c r="A5" s="2" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
     </row>
     <row r="6" spans="1:1">
       <c r="A6" s="2" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
     </row>
   </sheetData>
@@ -1590,37 +1608,37 @@
     </row>
     <row r="2" spans="1:1">
       <c r="A2" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="3" spans="1:1">
       <c r="A3" s="2" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
     </row>
     <row r="4" spans="1:1">
       <c r="A4" s="2" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
     </row>
     <row r="5" spans="1:1">
       <c r="A5" s="2" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
     </row>
     <row r="6" spans="1:1">
       <c r="A6" s="2" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
     </row>
     <row r="7" spans="1:1">
       <c r="A7" s="2" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
     </row>
     <row r="8" spans="1:1">
       <c r="A8" s="2" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
     </row>
   </sheetData>

</xml_diff>